<commit_message>
Devis : pages supplémentaires, commande en ligne, ajustements des options Shopify
- Option « Page supplémentaire » (30 € par page) avec libellés selon le domaine
  (services, plats, hébergements, formations, cours)
- Option « Commande en ligne (livraison ou à emporter) » à 290 € pour la restauration,
  les métiers de bouche, les producteurs locaux, les fleuristes et le pressing
- Shopify : retrait en magasin et cartes cadeaux inclus dans l'offre, relance de panier
  et Google Shopping + Meta Shop retirés, « Configuration de la livraison » à 90 €,
  multi-devises à 120 €, descriptions précisées
- Grille d'options et pages supplémentaires par domaine en Excel

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/grille-tarifaire-options.xlsx
+++ b/grille-tarifaire-options.xlsx
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -552,253 +552,285 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Réservation en ligne</t>
+          <t>Page supplémentaire</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Formulaire de réservation en ligne (rendez-vous, table, séance) avec créneaux et e-mails de confirmation</t>
+          <t>Au-delà des 3 pages de services incluses : une page dédiée (service, formation, plat…)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>140</v>
+        <v>30</v>
       </c>
       <c r="D6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Réservation avec acompte</t>
+          <t>Réservation en ligne</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Réservation + paiement en ligne (Stripe / PayPal)</t>
+          <t>Formulaire de réservation en ligne (rendez-vous, table, séance) avec créneaux et e-mails de confirmation</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>280</v>
+        <v>140</v>
       </c>
       <c r="D7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Formulaire de contact avancé</t>
+          <t>Réservation avec acompte</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Champs personnalisés, pièces jointes, anti-spam</t>
+          <t>Réservation + paiement en ligne (Stripe / PayPal)</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>60</v>
+        <v>280</v>
       </c>
       <c r="D8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Formulaire de devis élaboré</t>
+          <t>Commande en ligne (livraison ou à emporter)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Demande de devis en plusieurs étapes</t>
+          <t>Module de commande : carte en ligne, livraison ou à emporter, créneaux, paiement en ligne, notification des commandes</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>160</v>
+        <v>290</v>
       </c>
       <c r="D9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Bouton WhatsApp</t>
+          <t>Formulaire de contact avancé</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Bouton flottant avec message pré-rempli</t>
+          <t>Champs personnalisés, pièces jointes, anti-spam</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Pop-up promotionnelle</t>
+          <t>Formulaire de devis élaboré</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Pop-up ou bannière d'offre (promo, soldes, newsletter), ciblage et durée</t>
+          <t>Demande de devis en plusieurs étapes</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>60</v>
+        <v>160</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Newsletter</t>
+          <t>Bouton WhatsApp</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Inscription + connexion Mailchimp / Brevo</t>
+          <t>Bouton flottant avec message pré-rempli</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="D12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Blog</t>
+          <t>Pop-up promotionnelle</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Mise en page, catégories, partage</t>
+          <t>Pop-up ou bannière d'offre (promo, soldes, newsletter), ciblage et durée</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="D13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Article de blog (par article)</t>
+          <t>Newsletter</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Rédaction optimisée SEO (≈ 800 mots), images et mise en ligne</t>
+          <t>Inscription + connexion Mailchimp / Brevo</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="D14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Langue supplémentaire</t>
+          <t>Blog</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Traduction et sélecteur de langue (par langue)</t>
+          <t>Mise en page, catégories, partage</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>180</v>
+        <v>110</v>
       </c>
       <c r="D15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Avis clients</t>
+          <t>Article de blog (par article)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Affichage des avis Google sur le site</t>
+          <t>Rédaction optimisée SEO (≈ 800 mots), images et mise en ligne</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Mini boutique (≤ 20 produits)</t>
+          <t>Langue supplémentaire</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>WooCommerce : panier, paiement, livraison</t>
+          <t>Traduction et sélecteur de langue (par langue)</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>350</v>
+        <v>180</v>
       </c>
       <c r="D17" s="7" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>Avis clients</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Affichage des avis Google sur le site</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>90</v>
+      </c>
+      <c r="D18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Mini boutique (≤ 20 produits)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>WooCommerce : panier, paiement, livraison</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>350</v>
+      </c>
+      <c r="D19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
           <t>Espace membre</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Inscription, connexion, contenu réservé</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C20" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="D18" s="7" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="D20" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Offre de base</t>
         </is>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C22" s="9" t="n">
         <v>590</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Options choisies</t>
         </is>
       </c>
-      <c r="C21" s="10">
-        <f>SUMIF(D5:D18,"x",C5:C18)</f>
+      <c r="C23" s="10">
+        <f>SUMIF(D5:D20,"x",C5:C20)</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>TOTAL TTC</t>
         </is>
       </c>
-      <c r="B22" s="12" t="n"/>
-      <c r="C22" s="13">
-        <f>C20+C21</f>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="13">
+        <f>C22+C23</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Les licences d'extensions / applications payantes éventuelles sont facturées au coût réel. Prix modifiables (texte bleu).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Source : lib/pricing.ts du site (mêmes libellés et prix que la page /tarifs et le devis en ligne).</t>
         </is>
@@ -806,7 +838,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
   </dataValidations>
@@ -820,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -884,12 +916,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Paniers abandonnés</t>
+          <t>Ventes additionnelles</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>E-mails de relance automatiques</t>
+          <t>Packs, offres au panier et produits complémentaires (application dédiée)</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
@@ -900,269 +932,205 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Ventes additionnelles</t>
+          <t>Programme de fidélité</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Produits complémentaires et packs au panier</t>
+          <t>Points, récompenses, parrainage</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="D7" s="7" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Programme de fidélité</t>
+          <t>Abonnement produit</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Points, récompenses, parrainage</t>
+          <t>Plans d'abonnement (ex. mensuel), gestion et e-mails dédiés</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="D8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Abonnement produit</t>
+          <t>Précommande</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Vente récurrente (ex. mensuelle)</t>
+          <t>Parcours complet : message, date de livraison, alerte retour en stock</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="D9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Précommande</t>
+          <t>Produit personnalisable</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Vente avant stock + alerte retour en stock</t>
+          <t>Gravure, texte, options au choix</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>110</v>
+        <v>180</v>
       </c>
       <c r="D10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Produit personnalisable</t>
+          <t>Configuration de la livraison</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Gravure, texte, options au choix</t>
+          <t>Tarifs par zone et au poids, étiquettes et points relais Colissimo / Mondial Relay (Shopify Shipping)</t>
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="D11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Livraison avancée</t>
+          <t>Paiement en plusieurs fois</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Zones, tarifs au poids, Colissimo / Mondial Relay</t>
+          <t>Activation et intégration d'Alma / Klarna / PayPal 4x</t>
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="D12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Retrait en magasin</t>
+          <t>Multi-devises</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Click &amp; collect avec créneaux</t>
+          <t>Marchés internationaux : prix, taxes et devises par pays</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D13" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Paiement en plusieurs fois</t>
+          <t>Pack e-mailing</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Alma / Klarna / PayPal 4x</t>
+          <t>Bienvenue, post-achat, newsletter (Klaviyo)</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>60</v>
+        <v>210</v>
       </c>
       <c r="D14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Multi-devises</t>
+          <t>Blog boutique</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Prix et taxes par pays</t>
+          <t>Mise en page + SEO des articles</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="D15" s="7" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Cartes cadeaux</t>
+          <t>Import de produits (≤ 100)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Configuration + e-mail personnalisé</t>
+          <t>Import CSV, nettoyage et optimisation des fiches produit</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="D16" s="7" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Pack e-mailing</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Bienvenue, post-achat, newsletter (Klaviyo)</t>
-        </is>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>210</v>
-      </c>
-      <c r="D17" s="7" t="n"/>
-    </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Google Shopping + Meta Shop</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Catalogue connecté + pixels de suivi</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>140</v>
-      </c>
-      <c r="D18" s="7" t="n"/>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Offre de base</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>590</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Blog boutique</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Mise en page + SEO des articles</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>90</v>
-      </c>
-      <c r="D19" s="7" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Options choisies</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <f>SUMIF(D5:D16,"x",C5:C16)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Import de produits (≤ 100)</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Import CSV et optimisation des fiches</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n">
-        <v>140</v>
-      </c>
-      <c r="D20" s="7" t="n"/>
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL TTC</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="13">
+        <f>C18+C19</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Offre de base</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v>590</v>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Les licences d'extensions / applications payantes éventuelles sont facturées au coût réel. Prix modifiables (texte bleu).</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Options choisies</t>
-        </is>
-      </c>
-      <c r="C23" s="10">
-        <f>SUMIF(D5:D20,"x",C5:C20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL TTC</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="13">
-        <f>C22+C23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Les licences d'extensions / applications payantes éventuelles sont facturées au coût réel. Prix modifiables (texte bleu).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Source : lib/pricing.ts du site (mêmes libellés et prix que la page /tarifs et le devis en ligne).</t>
         </is>
@@ -1170,7 +1138,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>